<commit_message>
Update 2.4.2 Detection Benchmark Result
</commit_message>
<xml_diff>
--- a/tests/perf_v2/perf_history/v2.4.2/detection/DETECTION-aggregated.xlsx
+++ b/tests/perf_v2/perf_history/v2.4.2/detection/DETECTION-aggregated.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC12"/>
+  <dimension ref="A1:AC13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1714,6 +1714,109 @@
         </is>
       </c>
       <c r="AC12" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>yolox_x</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>769.4355</v>
+      </c>
+      <c r="C13" t="n">
+        <v>83.54470000000001</v>
+      </c>
+      <c r="D13" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4.3359</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.3656</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.0047</v>
+      </c>
+      <c r="H13" t="n">
+        <v>7.806</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.2211</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.9487</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.0036</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.9484</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.9441000000000001</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.1594</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.0021</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0.4378</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0.0065</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0.3774</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0.0056</v>
+      </c>
+      <c r="V13" t="n">
+        <v>20.0014</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.2971</v>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>2.4.2</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>DETECTION</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>Vitens-Aeromonas</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>eugene/benchmark/2.4.2</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>b7a58e7dd</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
@@ -3127,7 +3230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC12"/>
+  <dimension ref="A1:AC13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3486,74 +3589,74 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>rtdetr_101</t>
+          <t>dfine_x</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6285.4516</v>
+        <v>6618.7172</v>
       </c>
       <c r="C4" t="n">
-        <v>929.7348</v>
+        <v>2480.9224</v>
       </c>
       <c r="D4" t="n">
-        <v>45</v>
+        <v>52.8</v>
       </c>
       <c r="E4" t="n">
-        <v>7</v>
+        <v>19.4859</v>
       </c>
       <c r="F4" t="n">
-        <v>0.3154</v>
+        <v>0.5494</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0017</v>
+        <v>0.0031</v>
       </c>
       <c r="H4" t="n">
-        <v>17.34</v>
+        <v>17.724</v>
       </c>
       <c r="I4" t="n">
-        <v>0.8892</v>
+        <v>1.1422</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5937</v>
+        <v>0.5831</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0038</v>
+        <v>0.0271</v>
       </c>
       <c r="L4" t="n">
-        <v>0.5941</v>
+        <v>0.5838</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0035</v>
+        <v>0.0271</v>
       </c>
       <c r="N4" t="n">
-        <v>0.587</v>
+        <v>0.5787</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0048</v>
+        <v>0.0273</v>
       </c>
       <c r="P4" t="n">
-        <v>0.0568</v>
+        <v>0.0514</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0008</v>
+        <v>0.0009</v>
       </c>
       <c r="R4" t="n">
-        <v>0.2121</v>
+        <v>0.1796</v>
       </c>
       <c r="S4" t="n">
-        <v>0.0007</v>
+        <v>0.0016</v>
       </c>
       <c r="T4" t="n">
-        <v>0.126</v>
+        <v>0.1145</v>
       </c>
       <c r="U4" t="n">
-        <v>0.0004</v>
+        <v>0.0009</v>
       </c>
       <c r="V4" t="n">
-        <v>37.7952</v>
+        <v>34.3423</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1251</v>
+        <v>0.2745</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -3572,12 +3675,12 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>eugene/2.4.2-det-benchmark</t>
+          <t>eugene/benchmark/2.4.2</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>f3410bbc1</t>
+          <t>b7a58e7dd</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -3589,74 +3692,74 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>rtdetr_18</t>
+          <t>rtdetr_101</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8516.357099999999</v>
+        <v>6285.4516</v>
       </c>
       <c r="C5" t="n">
-        <v>1249.4537</v>
+        <v>929.7348</v>
       </c>
       <c r="D5" t="n">
-        <v>67.59999999999999</v>
+        <v>45</v>
       </c>
       <c r="E5" t="n">
-        <v>10.2127</v>
+        <v>7</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2854</v>
+        <v>0.3154</v>
       </c>
       <c r="G5" t="n">
-        <v>0.005</v>
+        <v>0.0017</v>
       </c>
       <c r="H5" t="n">
-        <v>8.029999999999999</v>
+        <v>17.34</v>
       </c>
       <c r="I5" t="n">
-        <v>0.3791</v>
+        <v>0.8892</v>
       </c>
       <c r="J5" t="n">
-        <v>0.5565</v>
+        <v>0.5937</v>
       </c>
       <c r="K5" t="n">
-        <v>0.003</v>
+        <v>0.0038</v>
       </c>
       <c r="L5" t="n">
-        <v>0.5563</v>
+        <v>0.5941</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0033</v>
+        <v>0.0035</v>
       </c>
       <c r="N5" t="n">
-        <v>0.5455</v>
+        <v>0.587</v>
       </c>
       <c r="O5" t="n">
-        <v>0.0046</v>
+        <v>0.0048</v>
       </c>
       <c r="P5" t="n">
-        <v>0.0456</v>
+        <v>0.0568</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0008</v>
       </c>
       <c r="R5" t="n">
-        <v>0.0885</v>
+        <v>0.2121</v>
       </c>
       <c r="S5" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0007</v>
       </c>
       <c r="T5" t="n">
-        <v>0.0762</v>
+        <v>0.126</v>
       </c>
       <c r="U5" t="n">
-        <v>0.0005</v>
+        <v>0.0004</v>
       </c>
       <c r="V5" t="n">
-        <v>22.8528</v>
+        <v>37.7952</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1625</v>
+        <v>0.1251</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
@@ -3692,74 +3795,74 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rtdetr_50</t>
+          <t>rtdetr_18</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5543.7777</v>
+        <v>8516.357099999999</v>
       </c>
       <c r="C6" t="n">
-        <v>846.8200000000001</v>
+        <v>1249.4537</v>
       </c>
       <c r="D6" t="n">
-        <v>43.8</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="E6" t="n">
-        <v>6.6858</v>
+        <v>10.2127</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2799</v>
+        <v>0.2854</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0031</v>
+        <v>0.005</v>
       </c>
       <c r="H6" t="n">
-        <v>14.59</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>0.8072</v>
+        <v>0.3791</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5904</v>
+        <v>0.5565</v>
       </c>
       <c r="K6" t="n">
-        <v>0.0072</v>
+        <v>0.003</v>
       </c>
       <c r="L6" t="n">
-        <v>0.5908</v>
+        <v>0.5563</v>
       </c>
       <c r="M6" t="n">
-        <v>0.007</v>
+        <v>0.0033</v>
       </c>
       <c r="N6" t="n">
-        <v>0.5762</v>
+        <v>0.5455</v>
       </c>
       <c r="O6" t="n">
-        <v>0.0061</v>
+        <v>0.0046</v>
       </c>
       <c r="P6" t="n">
-        <v>0.0501</v>
+        <v>0.0456</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.0015</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="R6" t="n">
-        <v>0.135</v>
+        <v>0.0885</v>
       </c>
       <c r="S6" t="n">
-        <v>0.0007</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="T6" t="n">
-        <v>0.1052</v>
+        <v>0.0762</v>
       </c>
       <c r="U6" t="n">
-        <v>0.0019</v>
+        <v>0.0005</v>
       </c>
       <c r="V6" t="n">
-        <v>31.5697</v>
+        <v>22.8528</v>
       </c>
       <c r="W6" t="n">
-        <v>0.5714</v>
+        <v>0.1625</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
@@ -3795,74 +3898,74 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>rtmdet_tiny</t>
+          <t>rtdetr_50</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5120.794</v>
+        <v>5543.7777</v>
       </c>
       <c r="C7" t="n">
-        <v>1147.3059</v>
+        <v>846.8200000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>72.8</v>
+        <v>43.8</v>
       </c>
       <c r="E7" t="n">
-        <v>16.2696</v>
+        <v>6.6858</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2297</v>
+        <v>0.2799</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0018</v>
+        <v>0.0031</v>
       </c>
       <c r="H7" t="n">
-        <v>4.182</v>
+        <v>14.59</v>
       </c>
       <c r="I7" t="n">
-        <v>0.2963</v>
+        <v>0.8072</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4437</v>
+        <v>0.5904</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0039</v>
+        <v>0.0072</v>
       </c>
       <c r="L7" t="n">
-        <v>0.4454</v>
+        <v>0.5908</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0034</v>
+        <v>0.007</v>
       </c>
       <c r="N7" t="n">
-        <v>0.4432</v>
+        <v>0.5762</v>
       </c>
       <c r="O7" t="n">
-        <v>0.0042</v>
+        <v>0.0061</v>
       </c>
       <c r="P7" t="n">
-        <v>0.0389</v>
+        <v>0.0501</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.0009</v>
+        <v>0.0015</v>
       </c>
       <c r="R7" t="n">
-        <v>0.0569</v>
+        <v>0.135</v>
       </c>
       <c r="S7" t="n">
-        <v>0.001</v>
+        <v>0.0007</v>
       </c>
       <c r="T7" t="n">
-        <v>0.0561</v>
+        <v>0.1052</v>
       </c>
       <c r="U7" t="n">
-        <v>0.0005</v>
+        <v>0.0019</v>
       </c>
       <c r="V7" t="n">
-        <v>16.8182</v>
+        <v>31.5697</v>
       </c>
       <c r="W7" t="n">
-        <v>0.1627</v>
+        <v>0.5714</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
@@ -3898,74 +4001,74 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ssd_mobilenetv2</t>
+          <t>rtmdet_tiny</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3959.5607</v>
+        <v>5120.794</v>
       </c>
       <c r="C8" t="n">
-        <v>1312.9736</v>
+        <v>1147.3059</v>
       </c>
       <c r="D8" t="n">
-        <v>58.4</v>
+        <v>72.8</v>
       </c>
       <c r="E8" t="n">
-        <v>19.9324</v>
+        <v>16.2696</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2624</v>
+        <v>0.2297</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0038</v>
+        <v>0.0018</v>
       </c>
       <c r="H8" t="n">
-        <v>6.29</v>
+        <v>4.182</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0212</v>
+        <v>0.2963</v>
       </c>
       <c r="J8" t="n">
-        <v>0.4229</v>
+        <v>0.4437</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0156</v>
+        <v>0.0039</v>
       </c>
       <c r="L8" t="n">
-        <v>0.4239</v>
+        <v>0.4454</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0156</v>
+        <v>0.0034</v>
       </c>
       <c r="N8" t="n">
-        <v>0.4235</v>
+        <v>0.4432</v>
       </c>
       <c r="O8" t="n">
-        <v>0.0155</v>
+        <v>0.0042</v>
       </c>
       <c r="P8" t="n">
-        <v>0.0365</v>
+        <v>0.0389</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.0013</v>
+        <v>0.0009</v>
       </c>
       <c r="R8" t="n">
-        <v>0.06279999999999999</v>
+        <v>0.0569</v>
       </c>
       <c r="S8" t="n">
-        <v>0.0015</v>
+        <v>0.001</v>
       </c>
       <c r="T8" t="n">
         <v>0.0561</v>
       </c>
       <c r="U8" t="n">
-        <v>0.0009</v>
+        <v>0.0005</v>
       </c>
       <c r="V8" t="n">
-        <v>16.8276</v>
+        <v>16.8182</v>
       </c>
       <c r="W8" t="n">
-        <v>0.2732</v>
+        <v>0.1627</v>
       </c>
       <c r="X8" t="inlineStr">
         <is>
@@ -4001,74 +4104,74 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>yolox_l</t>
+          <t>ssd_mobilenetv2</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4387.0593</v>
+        <v>3959.5607</v>
       </c>
       <c r="C9" t="n">
-        <v>582.8689000000001</v>
+        <v>1312.9736</v>
       </c>
       <c r="D9" t="n">
-        <v>59.4</v>
+        <v>58.4</v>
       </c>
       <c r="E9" t="n">
-        <v>8.018700000000001</v>
+        <v>19.9324</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2859</v>
+        <v>0.2624</v>
       </c>
       <c r="G9" t="n">
-        <v>0.001</v>
+        <v>0.0038</v>
       </c>
       <c r="H9" t="n">
-        <v>12.026</v>
+        <v>6.29</v>
       </c>
       <c r="I9" t="n">
-        <v>1.223</v>
+        <v>0.0212</v>
       </c>
       <c r="J9" t="n">
-        <v>0.5475</v>
+        <v>0.4229</v>
       </c>
       <c r="K9" t="n">
-        <v>0.0058</v>
+        <v>0.0156</v>
       </c>
       <c r="L9" t="n">
-        <v>0.5469000000000001</v>
+        <v>0.4239</v>
       </c>
       <c r="M9" t="n">
-        <v>0.0038</v>
+        <v>0.0156</v>
       </c>
       <c r="N9" t="n">
-        <v>0.5434</v>
+        <v>0.4235</v>
       </c>
       <c r="O9" t="n">
-        <v>0.0037</v>
+        <v>0.0155</v>
       </c>
       <c r="P9" t="n">
-        <v>0.0439</v>
+        <v>0.0365</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.0008</v>
+        <v>0.0013</v>
       </c>
       <c r="R9" t="n">
-        <v>0.1329</v>
+        <v>0.06279999999999999</v>
       </c>
       <c r="S9" t="n">
-        <v>0.0007</v>
+        <v>0.0015</v>
       </c>
       <c r="T9" t="n">
-        <v>0.0776</v>
+        <v>0.0561</v>
       </c>
       <c r="U9" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0009</v>
       </c>
       <c r="V9" t="n">
-        <v>23.2834</v>
+        <v>16.8276</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1944</v>
+        <v>0.2732</v>
       </c>
       <c r="X9" t="inlineStr">
         <is>
@@ -4104,74 +4207,74 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>yolox_s</t>
+          <t>yolox_l</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4141.7788</v>
+        <v>4387.0593</v>
       </c>
       <c r="C10" t="n">
-        <v>786.646</v>
+        <v>582.8689000000001</v>
       </c>
       <c r="D10" t="n">
-        <v>67</v>
+        <v>59.4</v>
       </c>
       <c r="E10" t="n">
-        <v>13.3791</v>
+        <v>8.018700000000001</v>
       </c>
       <c r="F10" t="n">
-        <v>0.209</v>
+        <v>0.2859</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0018</v>
+        <v>0.001</v>
       </c>
       <c r="H10" t="n">
-        <v>8.279999999999999</v>
+        <v>12.026</v>
       </c>
       <c r="I10" t="n">
-        <v>1.4411</v>
+        <v>1.223</v>
       </c>
       <c r="J10" t="n">
-        <v>0.4804</v>
+        <v>0.5475</v>
       </c>
       <c r="K10" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.0058</v>
       </c>
       <c r="L10" t="n">
-        <v>0.4825</v>
+        <v>0.5469000000000001</v>
       </c>
       <c r="M10" t="n">
-        <v>0.0066</v>
+        <v>0.0038</v>
       </c>
       <c r="N10" t="n">
-        <v>0.4792</v>
+        <v>0.5434</v>
       </c>
       <c r="O10" t="n">
-        <v>0.0075</v>
+        <v>0.0037</v>
       </c>
       <c r="P10" t="n">
-        <v>0.0351</v>
+        <v>0.0439</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.0009</v>
+        <v>0.0008</v>
       </c>
       <c r="R10" t="n">
-        <v>0.0639</v>
+        <v>0.1329</v>
       </c>
       <c r="S10" t="n">
-        <v>0.001</v>
+        <v>0.0007</v>
       </c>
       <c r="T10" t="n">
-        <v>0.0602</v>
+        <v>0.0776</v>
       </c>
       <c r="U10" t="n">
-        <v>0.0009</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="V10" t="n">
-        <v>18.07</v>
+        <v>23.2834</v>
       </c>
       <c r="W10" t="n">
-        <v>0.2696</v>
+        <v>0.1944</v>
       </c>
       <c r="X10" t="inlineStr">
         <is>
@@ -4195,7 +4298,7 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>97feded0d</t>
+          <t>f3410bbc1</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
@@ -4207,74 +4310,74 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>yolox_tiny</t>
+          <t>yolox_s</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2915.2236</v>
+        <v>4141.7788</v>
       </c>
       <c r="C11" t="n">
-        <v>841.9246000000001</v>
+        <v>786.646</v>
       </c>
       <c r="D11" t="n">
-        <v>58.8</v>
+        <v>67</v>
       </c>
       <c r="E11" t="n">
-        <v>17.0206</v>
+        <v>13.3791</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1643</v>
+        <v>0.209</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0018</v>
       </c>
       <c r="H11" t="n">
-        <v>5.8</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6955</v>
+        <v>1.4411</v>
       </c>
       <c r="J11" t="n">
-        <v>0.3416</v>
+        <v>0.4804</v>
       </c>
       <c r="K11" t="n">
-        <v>0.0118</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="L11" t="n">
-        <v>0.3437</v>
+        <v>0.4825</v>
       </c>
       <c r="M11" t="n">
-        <v>0.0102</v>
+        <v>0.0066</v>
       </c>
       <c r="N11" t="n">
-        <v>0.3375</v>
+        <v>0.4792</v>
       </c>
       <c r="O11" t="n">
-        <v>0.0095</v>
+        <v>0.0075</v>
       </c>
       <c r="P11" t="n">
-        <v>0.0249</v>
+        <v>0.0351</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.0005</v>
+        <v>0.0009</v>
       </c>
       <c r="R11" t="n">
-        <v>0.0523</v>
+        <v>0.0639</v>
       </c>
       <c r="S11" t="n">
-        <v>0.0015</v>
+        <v>0.001</v>
       </c>
       <c r="T11" t="n">
-        <v>0.0514</v>
+        <v>0.0602</v>
       </c>
       <c r="U11" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0009</v>
       </c>
       <c r="V11" t="n">
-        <v>15.4216</v>
+        <v>18.07</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1689</v>
+        <v>0.2696</v>
       </c>
       <c r="X11" t="inlineStr">
         <is>
@@ -4298,7 +4401,7 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>f3410bbc1</t>
+          <t>97feded0d</t>
         </is>
       </c>
       <c r="AC11" t="inlineStr">
@@ -4310,101 +4413,204 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>yolox_tiny</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2915.2236</v>
+      </c>
+      <c r="C12" t="n">
+        <v>841.9246000000001</v>
+      </c>
+      <c r="D12" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="E12" t="n">
+        <v>17.0206</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.1643</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="H12" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.6955</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.3416</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.0118</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.3437</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.0102</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.3375</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.0249</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0.0523</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0.0514</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="V12" t="n">
+        <v>15.4216</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.1689</v>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>2.4.2</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>DETECTION</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>visdrone</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>eugene/2.4.2-det-benchmark</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>f3410bbc1</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>yolox_x</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B13" t="n">
         <v>4890.6945</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C13" t="n">
         <v>692.1781999999999</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D13" t="n">
         <v>50.8</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E13" t="n">
         <v>7.3959</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F13" t="n">
         <v>0.206</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G13" t="n">
         <v>0.0004</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H13" t="n">
         <v>11.836</v>
       </c>
-      <c r="I12" t="n">
+      <c r="I13" t="n">
         <v>1.1406</v>
       </c>
-      <c r="J12" t="n">
+      <c r="J13" t="n">
         <v>0.5655</v>
       </c>
-      <c r="K12" t="n">
+      <c r="K13" t="n">
         <v>0.0035</v>
       </c>
-      <c r="L12" t="n">
+      <c r="L13" t="n">
         <v>0.5658</v>
       </c>
-      <c r="M12" t="n">
+      <c r="M13" t="n">
         <v>0.0036</v>
       </c>
-      <c r="N12" t="n">
+      <c r="N13" t="n">
         <v>0.5623</v>
       </c>
-      <c r="O12" t="n">
+      <c r="O13" t="n">
         <v>0.0039</v>
       </c>
-      <c r="P12" t="n">
+      <c r="P13" t="n">
         <v>0.0547</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="Q13" t="n">
         <v>0.0012</v>
       </c>
-      <c r="R12" t="n">
+      <c r="R13" t="n">
         <v>0.2008</v>
       </c>
-      <c r="S12" t="n">
+      <c r="S13" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T12" t="n">
+      <c r="T13" t="n">
         <v>0.0973</v>
       </c>
-      <c r="U12" t="n">
+      <c r="U13" t="n">
         <v>0.001</v>
       </c>
-      <c r="V12" t="n">
+      <c r="V13" t="n">
         <v>29.177</v>
       </c>
-      <c r="W12" t="n">
+      <c r="W13" t="n">
         <v>0.3089</v>
       </c>
-      <c r="X12" t="inlineStr">
+      <c r="X13" t="inlineStr">
         <is>
           <t>2.4.2</t>
         </is>
       </c>
-      <c r="Y12" t="inlineStr">
+      <c r="Y13" t="inlineStr">
         <is>
           <t>DETECTION</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr">
+      <c r="Z13" t="inlineStr">
         <is>
           <t>visdrone</t>
         </is>
       </c>
-      <c r="AA12" t="inlineStr">
+      <c r="AA13" t="inlineStr">
         <is>
           <t>eugene/2.4.2-det-benchmark</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr">
+      <c r="AB13" t="inlineStr">
         <is>
           <t>f3410bbc1</t>
         </is>
       </c>
-      <c r="AC12" t="inlineStr">
+      <c r="AC13" t="inlineStr">
         <is>
           <t>large</t>
         </is>

</xml_diff>